<commit_message>
posted LibraryExample code and updated news
</commit_message>
<xml_diff>
--- a/CS320-Sp25-TutoringSchedule.xlsx
+++ b/CS320-Sp25-TutoringSchedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\cygwin64\home\donha\cs320-spring2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EAD1B56-B120-40A9-A17D-6320F9ACDA37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67F7B48A-9248-45DC-B036-251CE6389314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="21480" windowHeight="14265" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="23070" windowHeight="15105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="21">
   <si>
     <t>Name</t>
   </si>
@@ -79,9 +79,6 @@
     <t xml:space="preserve"> </t>
   </si>
   <si>
-    <t>&lt;TBD&gt; will be serving as the version control tutors for CS320, as they have extensive experience with Git, GitHub, and setting up version control for teams</t>
-  </si>
-  <si>
     <t>Feel free to contact any of the tutors/mentors via email to arrange times to meet other than those listed here.  Weekday evening availability means that the tutors/mentors indicated they are available to meet at that time - you MUST still contact the tutor/mentor to schedule time with them, preferably with at least 24 hour advance notice.   They will NOT be available if you do NOT contact them first.</t>
   </si>
   <si>
@@ -92,6 +89,15 @@
   </si>
   <si>
     <t>Fri (in-class)</t>
+  </si>
+  <si>
+    <t>Brandon Woodward</t>
+  </si>
+  <si>
+    <t>Emmet Larsen</t>
+  </si>
+  <si>
+    <t>Brandon and Emmet will also be serving as the version control tutors for CS320, as they have extensive experience with Git, GitHub, and setting up version control for teams</t>
   </si>
 </sst>
 </file>
@@ -335,7 +341,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -434,12 +440,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -801,7 +801,7 @@
     </row>
     <row r="2" spans="1:25" s="7" customFormat="1" ht="85.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="23" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B2" s="23"/>
       <c r="C2" s="23"/>
@@ -860,17 +860,17 @@
         <v>6</v>
       </c>
       <c r="B4" s="38" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C4" s="39"/>
       <c r="D4" s="2"/>
       <c r="E4" s="38" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F4" s="39"/>
       <c r="G4" s="2"/>
       <c r="H4" s="38" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I4" s="39"/>
       <c r="J4" s="1"/>
@@ -912,39 +912,53 @@
       </c>
     </row>
     <row r="6" spans="1:25" s="3" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="17"/>
+      <c r="A6" s="17" t="s">
+        <v>18</v>
+      </c>
       <c r="B6" s="20" t="s">
         <v>5</v>
       </c>
       <c r="C6" s="16"/>
       <c r="D6" s="4"/>
-      <c r="E6" s="40"/>
-      <c r="F6" s="40"/>
-      <c r="G6" s="41"/>
-      <c r="H6" s="40"/>
-      <c r="I6" s="40"/>
+      <c r="E6" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="F6" s="16"/>
+      <c r="G6" s="4"/>
+      <c r="H6" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="I6" s="16"/>
     </row>
     <row r="7" spans="1:25" s="3" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="17"/>
-      <c r="B7" s="40"/>
-      <c r="C7" s="40"/>
+      <c r="A7" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="16"/>
+      <c r="C7" s="20" t="s">
+        <v>5</v>
+      </c>
       <c r="D7" s="4"/>
-      <c r="E7" s="40"/>
-      <c r="F7" s="40"/>
-      <c r="G7" s="41"/>
-      <c r="H7" s="40"/>
-      <c r="I7" s="40"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="G7" s="4"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="20" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="8" spans="1:25" s="3" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="17"/>
-      <c r="B8" s="40"/>
-      <c r="C8" s="40"/>
+      <c r="B8" s="16"/>
+      <c r="C8" s="16"/>
       <c r="D8" s="4"/>
-      <c r="E8" s="40"/>
-      <c r="F8" s="40"/>
-      <c r="G8" s="41"/>
-      <c r="H8" s="40"/>
-      <c r="I8" s="40"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="16"/>
+      <c r="I8" s="16"/>
     </row>
     <row r="9" spans="1:25" s="3" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="17" t="s">
@@ -1015,20 +1029,28 @@
       <c r="F14" s="37"/>
     </row>
     <row r="15" spans="1:25" s="3" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="17"/>
+      <c r="A15" s="17" t="s">
+        <v>18</v>
+      </c>
       <c r="B15" s="16"/>
       <c r="C15" s="16"/>
       <c r="D15" s="16"/>
       <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
+      <c r="F15" s="20" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="16" spans="1:25" s="3" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="17"/>
+      <c r="A16" s="17" t="s">
+        <v>19</v>
+      </c>
       <c r="B16" s="16"/>
       <c r="C16" s="16"/>
       <c r="D16" s="16"/>
       <c r="E16" s="16"/>
-      <c r="F16" s="16"/>
+      <c r="F16" s="20" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="17" spans="1:16" s="3" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="18"/>
@@ -1096,7 +1118,7 @@
         <v>0</v>
       </c>
       <c r="B23" s="27" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C23" s="28"/>
       <c r="D23" s="28"/>
@@ -1107,7 +1129,9 @@
       <c r="I23" s="29"/>
     </row>
     <row r="24" spans="1:16" s="3" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="14"/>
+      <c r="A24" s="14" t="s">
+        <v>18</v>
+      </c>
       <c r="B24" s="30"/>
       <c r="C24" s="31"/>
       <c r="D24" s="31"/>
@@ -1118,7 +1142,9 @@
       <c r="I24" s="32"/>
     </row>
     <row r="25" spans="1:16" s="3" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="21"/>
+      <c r="A25" s="21" t="s">
+        <v>19</v>
+      </c>
       <c r="B25" s="33"/>
       <c r="C25" s="34"/>
       <c r="D25" s="34"/>

</xml_diff>